<commit_message>
Einkaufsliste: günstiger Korb mit Pololu S13V10F5 (Berrybase 9,95 €) statt MT3608 – MT3608 liefert bei 3,7 V nur ca. 0,5 A; Korb 84,10 € -> 92,01 €
</commit_message>
<xml_diff>
--- a/doku/Einkaufsliste_HydroDesk_guenstig.xlsx
+++ b/doku/Einkaufsliste_HydroDesk_guenstig.xlsx
@@ -2860,72 +2860,76 @@
       <c r="P23" s="35" t="n"/>
     </row>
     <row r="24" ht="28.35" customHeight="1" s="25">
-      <c r="A24" s="27" t="n">
+      <c r="A24" s="31" t="n">
         <v>8</v>
       </c>
-      <c r="B24" s="27" t="inlineStr">
+      <c r="B24" s="31" t="inlineStr">
         <is>
           <t>Step-Up 5 V</t>
         </is>
       </c>
-      <c r="C24" s="27" t="inlineStr">
+      <c r="C24" s="31" t="inlineStr">
         <is>
           <t>Berrybase</t>
         </is>
       </c>
-      <c r="D24" s="27" t="inlineStr">
+      <c r="D24" s="31" t="inlineStr">
         <is>
           <t>Pololu S13V10F5 5 V 1 A Step-Up/Step-Down</t>
         </is>
       </c>
-      <c r="E24" s="27" t="inlineStr">
+      <c r="E24" s="31" t="inlineStr">
         <is>
           <t>1 Stk</t>
         </is>
       </c>
-      <c r="F24" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="G24" s="28" t="n">
+      <c r="F24" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="32" t="n">
         <v>9.949999999999999</v>
       </c>
-      <c r="H24" s="29">
+      <c r="H24" s="33">
         <f>G24/F24</f>
         <v/>
       </c>
-      <c r="I24" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="J24" s="28">
+      <c r="I24" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="J24" s="32">
         <f>ROUNDUP(I24/F24,0)*G24</f>
         <v/>
       </c>
-      <c r="K24" s="27" t="inlineStr">
+      <c r="K24" s="31" t="inlineStr">
         <is>
           <t>4,95 € DHL, frei ab 150 €</t>
         </is>
       </c>
-      <c r="L24" s="27" t="inlineStr">
+      <c r="L24" s="31" t="inlineStr">
         <is>
           <t>1–3 Tage</t>
         </is>
       </c>
-      <c r="M24" s="30" t="inlineStr">
+      <c r="M24" s="34" t="inlineStr">
         <is>
           <t>https://www.berrybase.de/pololu-s13v10f5-5v-1a-step-up-step-down-converter</t>
         </is>
       </c>
-      <c r="N24" s="27" t="inlineStr">
+      <c r="N24" s="31" t="inlineStr">
         <is>
           <t>08.10.2026</t>
         </is>
       </c>
-      <c r="O24" s="27" t="inlineStr">
-        <is>
-          <t>EMPFOHLEN: fest 5 V, UVLO, Softstart, Überstromschutz; klein (ca. 9×12 mm) → im 37×17-Fach fixieren</t>
-        </is>
-      </c>
-      <c r="P24" s="27" t="n"/>
+      <c r="O24" s="31" t="inlineStr">
+        <is>
+          <t>GEWÄHLT in beiden Körben (08.10.2026): fest 5 V, 1 A, UVLO, Softstart, Überstromschutz; klein (ca. 9×12 mm) → im 37×17-Fach fixieren. Vergleich: Botland 7,90 € + Versand ab 4,99 € (eigener Shop, https://botland.de/aufwarts-abwartswandler/21022-s13v10f5-aufwarts-abwartswandler-5v-1a-pololu-4083.html), Eckstein 11,80 € – Berrybase ist im Korb am günstigsten, weil der Berrybase-Versand ohnehin anfällt</t>
+        </is>
+      </c>
+      <c r="P24" s="31" t="inlineStr">
+        <is>
+          <t>✔ günstigste</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="25">
       <c r="A25" s="27" t="n">
@@ -2996,76 +3000,72 @@
       <c r="P25" s="27" t="n"/>
     </row>
     <row r="26" ht="28.35" customHeight="1" s="25">
-      <c r="A26" s="31" t="n">
+      <c r="A26" s="35" t="n">
         <v>8</v>
       </c>
-      <c r="B26" s="31" t="inlineStr">
+      <c r="B26" s="35" t="inlineStr">
         <is>
           <t>Step-Up 5 V</t>
         </is>
       </c>
-      <c r="C26" s="31" t="inlineStr">
+      <c r="C26" s="35" t="inlineStr">
         <is>
           <t>AliExpress</t>
         </is>
       </c>
-      <c r="D26" s="31" t="inlineStr">
+      <c r="D26" s="35" t="inlineStr">
         <is>
           <t>MT3608 Step-Up einstellbar (2 Stk)</t>
         </is>
       </c>
-      <c r="E26" s="31" t="inlineStr">
+      <c r="E26" s="35" t="inlineStr">
         <is>
           <t>2 Stk</t>
         </is>
       </c>
-      <c r="F26" s="31" t="n">
+      <c r="F26" s="35" t="n">
         <v>2</v>
       </c>
-      <c r="G26" s="32" t="n">
+      <c r="G26" s="37" t="n">
         <v>2.04</v>
       </c>
-      <c r="H26" s="33">
+      <c r="H26" s="38">
         <f>G26/F26</f>
         <v/>
       </c>
-      <c r="I26" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="J26" s="32">
+      <c r="I26" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="J26" s="37">
         <f>ROUNDUP(I26/F26,0)*G26</f>
         <v/>
       </c>
-      <c r="K26" s="31" t="inlineStr">
+      <c r="K26" s="35" t="inlineStr">
         <is>
           <t>lt. Liste '3+, kein Zollaufschlag'</t>
         </is>
       </c>
-      <c r="L26" s="31" t="inlineStr">
+      <c r="L26" s="35" t="inlineStr">
         <is>
           <t>1–3 Wochen</t>
         </is>
       </c>
-      <c r="M26" s="34" t="inlineStr">
+      <c r="M26" s="36" t="inlineStr">
         <is>
           <t>https://de.aliexpress.com/item/1005009806778521.html</t>
         </is>
       </c>
-      <c r="N26" s="31" t="inlineStr">
+      <c r="N26" s="35" t="inlineStr">
         <is>
           <t>08.10.2026</t>
         </is>
       </c>
-      <c r="O26" s="31" t="inlineStr">
-        <is>
-          <t>NUR MIT VORSICHT: Poti vorher auf 5,0 V stellen; bei 3,7→5 V real ca. 0,5 A, Ripple, heiß</t>
-        </is>
-      </c>
-      <c r="P26" s="31" t="inlineStr">
-        <is>
-          <t>✔ günstigste</t>
-        </is>
-      </c>
+      <c r="O26" s="35" t="inlineStr">
+        <is>
+          <t>GESTRICHEN 08.10.2026 (auch im günstigen Korb): bei 3,7→5 V real nur ca. 0,5 A – zu wenig für CYD (0,25–0,35 A) + 26 COB-LEDs (bis ca. 0,49 A); Poti, Ripple, heiß</t>
+        </is>
+      </c>
+      <c r="P26" s="35" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1" s="25">
       <c r="A27" s="35" t="n">
@@ -3126,7 +3126,7 @@
       </c>
       <c r="O27" s="35" t="inlineStr">
         <is>
-          <t>derzeit nicht verfügbar</t>
+          <t>derzeit nicht verfügbar; außerdem zu schwach (siehe Zeile darüber)</t>
         </is>
       </c>
       <c r="P27" s="35" t="n"/>
@@ -5084,7 +5084,7 @@
       </c>
       <c r="I11" s="27" t="inlineStr">
         <is>
-          <t>empfohlen statt MT3608</t>
+          <t>statt MT3608 (zu schwach, ca. 0,5 A bei 3,7 V)</t>
         </is>
       </c>
     </row>
@@ -5781,19 +5781,19 @@
       </c>
       <c r="C35" s="27" t="inlineStr">
         <is>
-          <t>AliExpress</t>
+          <t>Berrybase</t>
         </is>
       </c>
       <c r="D35" s="27" t="inlineStr">
         <is>
-          <t>MT3608 2 Stk (ab-Preis)</t>
+          <t>Pololu S13V10F5 5 V 1 A</t>
         </is>
       </c>
       <c r="E35" s="27" t="n">
         <v>1</v>
       </c>
       <c r="F35" s="28" t="n">
-        <v>2.04</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="G35" s="28">
         <f>E35*F35</f>
@@ -5801,12 +5801,12 @@
       </c>
       <c r="H35" s="30" t="inlineStr">
         <is>
-          <t>https://de.aliexpress.com/item/1005009806778521.html</t>
+          <t>https://www.berrybase.de/pololu-s13v10f5-5v-1a-step-up-step-down-converter</t>
         </is>
       </c>
       <c r="I35" s="27" t="inlineStr">
         <is>
-          <t>nur mit Vorsicht – Upgrade Pololu +9,95 €</t>
+          <t>statt MT3608 (08.10.2026): MT3608 liefert bei 3,7 V nur ca. 0,5 A – zu wenig für CYD + 26 COB-LEDs</t>
         </is>
       </c>
     </row>

</xml_diff>